<commit_message>
Updating filtered feeds from workflow
</commit_message>
<xml_diff>
--- a/filtered_feeds.xlsx
+++ b/filtered_feeds.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="174">
   <si>
     <t>link</t>
   </si>
@@ -313,6 +313,18 @@
     <t>https://www.360dx.com/cancer/acrivon-therapeutics-open-clia-certified-lab-run-diagnostics-targeted-therapies</t>
   </si>
   <si>
+    <t>https://www.genomeweb.com/regulatory-news-fda-approvals/biocartis-gets-ivdr-certification-colorectal-cancer-cdx</t>
+  </si>
+  <si>
+    <t>https://www.genomeweb.com/cancer/foundation-medicine-expands-participation-nci-led-cancer-therapy-combination-initiative</t>
+  </si>
+  <si>
+    <t>https://www.360dx.com/regulatory-news-fda-approvals/biocartis-gets-ivdr-certification-colorectal-cancer-cdx</t>
+  </si>
+  <si>
+    <t>https://www.360dx.com/cancer/foundation-medicine-expands-participation-nci-led-cancer-therapy-combination-initiative</t>
+  </si>
+  <si>
     <t>companion diagnostic</t>
   </si>
   <si>
@@ -518,6 +530,12 @@
   </si>
   <si>
     <t>Acrivon Therapeutics to Open CLIA-Certified Lab to Run Diagnostics for Targeted Therapies</t>
+  </si>
+  <si>
+    <t>Biocartis Gets IVDR Certification for Colorectal Cancer CDx</t>
+  </si>
+  <si>
+    <t>Foundation Medicine Expands Participation in NCI-led Cancer Therapy Combination Initiative</t>
   </si>
 </sst>
 </file>
@@ -862,7 +880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="60.7109375" customWidth="1"/>
@@ -886,10 +904,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -897,10 +915,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -908,10 +926,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -919,10 +937,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -930,10 +948,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -941,10 +959,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -952,10 +970,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -963,10 +981,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -974,10 +992,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -985,10 +1003,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -996,10 +1014,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1007,10 +1025,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1018,10 +1036,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C14" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1029,10 +1047,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1040,10 +1058,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1051,10 +1069,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C17" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1062,10 +1080,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C18" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1073,10 +1091,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C19" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1084,10 +1102,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1095,10 +1113,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C21" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1106,10 +1124,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1117,10 +1135,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C23" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1128,10 +1146,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C24" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1139,10 +1157,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C25" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1150,10 +1168,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C26" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1161,10 +1179,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1172,10 +1190,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C28" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1183,10 +1201,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C29" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1194,10 +1212,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1205,10 +1223,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C31" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1216,10 +1234,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1227,10 +1245,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C33" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1238,10 +1256,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C34" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1249,10 +1267,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C35" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1260,10 +1278,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1271,10 +1289,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C37" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1282,10 +1300,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1293,10 +1311,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C39" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1304,10 +1322,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C40" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1315,10 +1333,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C41" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1326,10 +1344,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C42" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1337,10 +1355,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C43" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1348,10 +1366,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C44" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1359,10 +1377,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C45" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1370,10 +1388,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C46" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1381,10 +1399,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1392,10 +1410,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C48" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1403,10 +1421,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C49" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1414,10 +1432,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C50" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1425,10 +1443,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C51" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1436,10 +1454,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C52" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1447,10 +1465,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C53" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1458,10 +1476,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C54" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1469,10 +1487,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C55" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1480,10 +1498,10 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C56" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1491,10 +1509,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C57" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1502,10 +1520,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C58" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1513,10 +1531,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C59" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1524,10 +1542,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C60" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1535,10 +1553,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C61" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1546,10 +1564,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C62" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1557,10 +1575,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C63" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1568,10 +1586,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C64" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1579,10 +1597,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C65" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1590,10 +1608,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C66" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1601,10 +1619,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C67" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1612,10 +1630,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C68" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1623,10 +1641,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C69" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1634,10 +1652,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C70" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1645,10 +1663,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C71" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1656,10 +1674,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C72" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1667,10 +1685,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C73" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1678,10 +1696,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C74" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1689,10 +1707,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C75" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1700,10 +1718,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C76" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1711,10 +1729,10 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C77" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1722,10 +1740,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C78" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -1733,10 +1751,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C79" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -1744,10 +1762,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C80" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -1755,10 +1773,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C81" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -1766,10 +1784,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C82" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -1777,10 +1795,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C83" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -1788,10 +1806,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C84" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -1799,10 +1817,10 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C85" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -1810,10 +1828,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C86" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -1821,10 +1839,10 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C87" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -1832,10 +1850,10 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C88" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -1843,10 +1861,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C89" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -1854,10 +1872,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C90" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -1865,10 +1883,10 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C91" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -1876,10 +1894,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C92" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -1887,10 +1905,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C93" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -1898,10 +1916,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C94" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -1909,10 +1927,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C95" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -1920,10 +1938,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C96" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -1931,10 +1949,54 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
+        <v>104</v>
+      </c>
+      <c r="C97" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B98" t="s">
+        <v>104</v>
+      </c>
+      <c r="C98" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C97" t="s">
-        <v>167</v>
+      <c r="B99" t="s">
+        <v>104</v>
+      </c>
+      <c r="C99" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3">
+      <c r="A100" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B100" t="s">
+        <v>104</v>
+      </c>
+      <c r="C100" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3">
+      <c r="A101" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B101" t="s">
+        <v>104</v>
+      </c>
+      <c r="C101" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -2035,6 +2097,10 @@
     <hyperlink ref="A95" r:id="rId94"/>
     <hyperlink ref="A96" r:id="rId95"/>
     <hyperlink ref="A97" r:id="rId96"/>
+    <hyperlink ref="A98" r:id="rId97"/>
+    <hyperlink ref="A99" r:id="rId98"/>
+    <hyperlink ref="A100" r:id="rId99"/>
+    <hyperlink ref="A101" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>